<commit_message>
Regenerate preprocessing report for GNB targets
</commit_message>
<xml_diff>
--- a/mepram/preprocessing_report/tables/summary_excel_file.xlsx
+++ b/mepram/preprocessing_report/tables/summary_excel_file.xlsx
@@ -56,7 +56,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q419"/>
+  <dimension ref="A1:Q420"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -36097,7 +36097,7 @@
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>resultado_hemo_gbn_selected</t>
+          <t>resultado_hemo_gnb_selected</t>
         </is>
       </c>
       <c r="B415" t="inlineStr">
@@ -36162,7 +36162,7 @@
       </c>
       <c r="N415" t="inlineStr">
         <is>
-          <t>NEGATIVE: 53.0%; GBNSelected: 33.7%; other_etiology: 13.3%</t>
+          <t>NEGATIVE: 53.0%; GNBSelected: 33.7%; other_etiology: 13.3%</t>
         </is>
       </c>
       <c r="O415" t="inlineStr">
@@ -36184,7 +36184,7 @@
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>infected_yes_no</t>
+          <t>resultado_hemo_gnb_all</t>
         </is>
       </c>
       <c r="B416" t="inlineStr">
@@ -36204,7 +36204,7 @@
       </c>
       <c r="E416" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F416" t="inlineStr">
@@ -36234,7 +36234,7 @@
       </c>
       <c r="K416" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="L416" t="inlineStr">
@@ -36249,7 +36249,7 @@
       </c>
       <c r="N416" t="inlineStr">
         <is>
-          <t>NEGATIVE: 53.0%; POSITIVE: 47.0%</t>
+          <t>NEGATIVE: 53.0%; GNBAll: 34.6%; other_etiology: 12.5%</t>
         </is>
       </c>
       <c r="O416" t="inlineStr">
@@ -36271,7 +36271,7 @@
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>fenotipo_resistencia_individual</t>
+          <t>infected_yes_no</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
@@ -36291,12 +36291,12 @@
       </c>
       <c r="E417" t="inlineStr">
         <is>
-          <t>13 exploded labels; 75 row-level combinations</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t>tuple</t>
+          <t>string</t>
         </is>
       </c>
       <c r="G417" t="inlineStr">
@@ -36321,22 +36321,22 @@
       </c>
       <c r="K417" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>2</t>
         </is>
       </c>
       <c r="L417" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>NEGATIVE</t>
         </is>
       </c>
       <c r="M417" t="inlineStr">
         <is>
-          <t>80.6</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="N417" t="inlineStr">
         <is>
-          <t>[]: 80.6%; ['Bacilo Gram negativo resistente a amoxicilina/clavulánico']: 3.9%; ['Coco Gram positivo resistente a ampicilina o penicilina']: 2.5%</t>
+          <t>NEGATIVE: 53.0%; POSITIVE: 47.0%</t>
         </is>
       </c>
       <c r="O417" t="inlineStr">
@@ -36358,7 +36358,7 @@
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>resistente_cefalosporina</t>
+          <t>fenotipo_resistencia_individual</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
@@ -36378,12 +36378,12 @@
       </c>
       <c r="E418" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>13 exploded labels; 75 row-level combinations</t>
         </is>
       </c>
       <c r="F418" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>tuple</t>
         </is>
       </c>
       <c r="G418" t="inlineStr">
@@ -36408,22 +36408,22 @@
       </c>
       <c r="K418" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>75</t>
         </is>
       </c>
       <c r="L418" t="inlineStr">
         <is>
-          <t>NEGATIVE</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="M418" t="inlineStr">
         <is>
-          <t>94.0</t>
+          <t>80.6</t>
         </is>
       </c>
       <c r="N418" t="inlineStr">
         <is>
-          <t>NEGATIVE: 94.0%; RESIST_CEFALOSPORINAS_3a_4a: 6.0%</t>
+          <t>[]: 80.6%; ['Bacilo Gram negativo resistente a amoxicilina/clavulánico']: 3.9%; ['Coco Gram positivo resistente a ampicilina o penicilina']: 2.5%</t>
         </is>
       </c>
       <c r="O418" t="inlineStr">
@@ -36445,91 +36445,178 @@
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
+          <t>resistente_cefalosporina</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Predictive targets</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>target_building</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J419" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K419" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="L419" t="inlineStr">
+        <is>
+          <t>NEGATIVE</t>
+        </is>
+      </c>
+      <c r="M419" t="inlineStr">
+        <is>
+          <t>94.0</t>
+        </is>
+      </c>
+      <c r="N419" t="inlineStr">
+        <is>
+          <t>NEGATIVE: 94.0%; RESIST_CEFALOSPORINAS_3a_4a: 6.0%</t>
+        </is>
+      </c>
+      <c r="O419" t="inlineStr">
+        <is>
+          <t>Prediction target or target-support variable derived during target building.</t>
+        </is>
+      </c>
+      <c r="P419" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Q419" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
           <t>resistente_cefalosporina_multi</t>
         </is>
       </c>
-      <c r="B419" t="inlineStr">
+      <c r="B420" t="inlineStr">
         <is>
           <t>Predictive targets</t>
         </is>
       </c>
-      <c r="C419" t="inlineStr">
+      <c r="C420" t="inlineStr">
         <is>
           <t>target_building</t>
         </is>
       </c>
-      <c r="D419" t="inlineStr">
+      <c r="D420" t="inlineStr">
         <is>
           <t>target</t>
         </is>
       </c>
-      <c r="E419" t="inlineStr">
+      <c r="E420" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="F419" t="inlineStr">
+      <c r="F420" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="G419" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="H419" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I419" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J419" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K419" t="inlineStr">
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J420" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K420" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="L419" t="inlineStr">
+      <c r="L420" t="inlineStr">
         <is>
           <t>NEGATIVE</t>
         </is>
       </c>
-      <c r="M419" t="inlineStr">
+      <c r="M420" t="inlineStr">
         <is>
           <t>80.6</t>
         </is>
       </c>
-      <c r="N419" t="inlineStr">
+      <c r="N420" t="inlineStr">
         <is>
           <t>NEGATIVE: 80.6%; OTHER: 13.4%; RESIST_CEFALOSPORINAS_3a_4a: 6.0%</t>
         </is>
       </c>
-      <c r="O419" t="inlineStr">
+      <c r="O420" t="inlineStr">
         <is>
           <t>Prediction target or target-support variable derived during target building.</t>
         </is>
       </c>
-      <c r="P419" t="inlineStr">
+      <c r="P420" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="Q419" t="inlineStr">
+      <c r="Q420" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q419"/>
+  <autoFilter ref="A1:Q420"/>
 </worksheet>
 </file>
</xml_diff>